<commit_message>
add dummy values for missing investment cost
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/investment_cost_overview/investment_cost_overview.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/investment_cost_overview/investment_cost_overview.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/djh_eco_cbs_dk/Documents/Documents/GitHub/Nord_H2ub/Spine_Projects/01_input_data/01_input_raw/investment_cost_overview/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\investment_cost_overview\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{6D0F3777-73D1-41BF-80D4-5E66D841CD10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A7A42DF-DD73-4FE7-A1B4-256E7DE21FF2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FB704F-99AD-4337-A42C-1D101EB4274B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{B319F6F4-5B26-4633-9938-205A8FCCCA95}"/>
+    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{B319F6F4-5B26-4633-9938-205A8FCCCA95}"/>
   </bookViews>
   <sheets>
     <sheet name="Investment_Cost" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentManualCount="6"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="51">
   <si>
     <t>PV_plant</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t>Power_storage</t>
+  </si>
+  <si>
+    <t>dummy values</t>
   </si>
 </sst>
 </file>
@@ -744,16 +747,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FABD746-4A8E-4371-B5EF-19107F5A398A}">
   <dimension ref="A1:I29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="32.26953125" customWidth="1"/>
-    <col min="7" max="7" width="10.08984375" customWidth="1"/>
-    <col min="8" max="8" width="16.54296875" customWidth="1"/>
+    <col min="1" max="1" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="32.21875" customWidth="1"/>
+    <col min="7" max="7" width="10.109375" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" customWidth="1"/>
     <col min="9" max="9" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -782,7 +785,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -809,7 +812,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -836,7 +839,7 @@
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -863,7 +866,7 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -890,7 +893,7 @@
       </c>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -917,7 +920,7 @@
       </c>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -944,7 +947,7 @@
       </c>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -971,7 +974,7 @@
       </c>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -998,7 +1001,7 @@
       </c>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1025,7 +1028,7 @@
       </c>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1052,7 +1055,7 @@
       </c>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1079,7 +1082,7 @@
       </c>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1106,7 +1109,7 @@
       </c>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>36</v>
       </c>
@@ -1133,7 +1136,7 @@
       </c>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -1160,7 +1163,7 @@
       </c>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -1187,7 +1190,7 @@
       </c>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1216,7 +1219,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1243,7 +1246,7 @@
       </c>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -1272,7 +1275,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1299,7 +1302,7 @@
       </c>
       <c r="I20" s="4"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1326,7 +1329,7 @@
       </c>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1352,43 +1355,94 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="4"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B23" s="4">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4">
+        <v>1</v>
+      </c>
+      <c r="D23" s="4">
+        <v>1</v>
+      </c>
+      <c r="E23" s="4">
+        <v>1</v>
+      </c>
+      <c r="F23" s="4">
+        <v>1</v>
+      </c>
+      <c r="G23" t="s">
+        <v>22</v>
+      </c>
+      <c r="H23" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="4"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B24" s="4">
+        <v>1</v>
+      </c>
+      <c r="C24" s="4">
+        <v>1</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1</v>
+      </c>
+      <c r="E24" s="4">
+        <v>1</v>
+      </c>
+      <c r="F24" s="4">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="I24" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="4"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B25" s="4">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4">
+        <v>1</v>
+      </c>
+      <c r="D25" s="4">
+        <v>1</v>
+      </c>
+      <c r="E25" s="4">
+        <v>1</v>
+      </c>
+      <c r="F25" s="4">
+        <v>1</v>
+      </c>
+      <c r="G25" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>42</v>
       </c>
@@ -1407,12 +1461,17 @@
       <c r="F26" s="4">
         <v>4400</v>
       </c>
-      <c r="H26" s="5"/>
+      <c r="G26" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="5">
+        <v>0.05</v>
+      </c>
       <c r="I26" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>49</v>
       </c>
@@ -1431,10 +1490,17 @@
       <c r="F27" s="4">
         <v>1</v>
       </c>
-      <c r="H27" s="5"/>
-      <c r="I27" s="4"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="G27" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="5">
+        <v>0.05</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -1443,7 +1509,7 @@
       <c r="H28" s="5"/>
       <c r="I28" s="4"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -1464,19 +1530,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262416F5-07F9-4A10-AA36-6136A8834922}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -1484,7 +1550,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>

</xml_diff>